<commit_message>
Correccion de formatos de carga y subida y editar plantilla
</commit_message>
<xml_diff>
--- a/resources/formatos/FormatoCeldas.xlsx
+++ b/resources/formatos/FormatoCeldas.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\xampp\htdocs\E-Monitoring-SqlServer\resources\formatos\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\laragon\www\E-Monitoring-SqlServer\resources\formatos\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8E8A5E33-0375-4F20-BC26-BF374D7D64B9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91BBC1B5-C417-4C02-9CAA-65DCCF6E045C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Celdas" sheetId="1" r:id="rId1"/>
@@ -36,18 +36,12 @@
     <t>Nombre:</t>
   </si>
   <si>
-    <t>Cota Instalación (m.s.n.m):</t>
-  </si>
-  <si>
     <t>C.F.:</t>
   </si>
   <si>
     <t>Marca:</t>
   </si>
   <si>
-    <t>Cota Fundación (m.s.n.m):</t>
-  </si>
-  <si>
     <t>T.K.:</t>
   </si>
   <si>
@@ -63,9 +57,6 @@
     <t>Hora</t>
   </si>
   <si>
-    <t>Frecuencia (Digits)</t>
-  </si>
-  <si>
     <t>Frecuencia (Hz)</t>
   </si>
   <si>
@@ -81,15 +72,9 @@
     <t>FORMATO DE DATOS - CELDAS DE ASENTAMIENTO</t>
   </si>
   <si>
-    <t>Desplazamiento (m)</t>
-  </si>
-  <si>
     <t>Rango (m):</t>
   </si>
   <si>
-    <t>Cota de Superficie Actual (m.s.n.m):</t>
-  </si>
-  <si>
     <t>Coordenada Este (m):</t>
   </si>
   <si>
@@ -112,6 +97,21 @@
   </si>
   <si>
     <t>* El formato de hora: hh:mm:ss</t>
+  </si>
+  <si>
+    <t>Cota Instalación (msnm):</t>
+  </si>
+  <si>
+    <t>Cota Fundación (msnm):</t>
+  </si>
+  <si>
+    <t>Cota de Superficie Actual (msnm):</t>
+  </si>
+  <si>
+    <t>Frecuencia (digits)</t>
+  </si>
+  <si>
+    <t>Asentamiento (m)</t>
   </si>
 </sst>
 </file>
@@ -437,28 +437,43 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
@@ -470,44 +485,29 @@
     <xf numFmtId="0" fontId="0" fillId="3" borderId="9" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="4" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="6" xfId="0" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="20" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="15" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="20" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -854,215 +854,215 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:G16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.90625" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="7" width="20" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="23"/>
-      <c r="B1" s="26" t="s">
-        <v>17</v>
-      </c>
-      <c r="C1" s="27"/>
-      <c r="D1" s="27"/>
-      <c r="E1" s="27"/>
-      <c r="F1" s="27"/>
-      <c r="G1" s="28"/>
-    </row>
-    <row r="2" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="24"/>
-      <c r="B2" s="29"/>
-      <c r="C2" s="30"/>
-      <c r="D2" s="30"/>
-      <c r="E2" s="30"/>
-      <c r="F2" s="30"/>
-      <c r="G2" s="31"/>
-    </row>
-    <row r="3" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="24"/>
-      <c r="B3" s="32" t="s">
-        <v>27</v>
-      </c>
-      <c r="C3" s="33"/>
-      <c r="D3" s="33"/>
-      <c r="E3" s="33"/>
-      <c r="F3" s="33"/>
-      <c r="G3" s="34"/>
-    </row>
-    <row r="4" spans="1:7" ht="25" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A4" s="25"/>
-      <c r="B4" s="32" t="s">
-        <v>28</v>
-      </c>
-      <c r="C4" s="33"/>
-      <c r="D4" s="33"/>
-      <c r="E4" s="33"/>
-      <c r="F4" s="33"/>
-      <c r="G4" s="34"/>
-    </row>
-    <row r="5" spans="1:7" ht="14.4" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A5" s="5"/>
-      <c r="B5" s="6"/>
-      <c r="C5" s="6"/>
-      <c r="D5" s="6"/>
-      <c r="E5" s="6"/>
-      <c r="F5" s="6"/>
-      <c r="G5" s="7"/>
-    </row>
-    <row r="6" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A6" s="22" t="s">
-        <v>0</v>
-      </c>
-      <c r="B6" s="17"/>
-      <c r="C6" s="18"/>
-      <c r="D6" s="16" t="s">
+    <row r="1" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A1" s="5"/>
+      <c r="B1" s="8" t="s">
+        <v>14</v>
+      </c>
+      <c r="C1" s="9"/>
+      <c r="D1" s="9"/>
+      <c r="E1" s="9"/>
+      <c r="F1" s="9"/>
+      <c r="G1" s="10"/>
+    </row>
+    <row r="2" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A2" s="6"/>
+      <c r="B2" s="11"/>
+      <c r="C2" s="12"/>
+      <c r="D2" s="12"/>
+      <c r="E2" s="12"/>
+      <c r="F2" s="12"/>
+      <c r="G2" s="13"/>
+    </row>
+    <row r="3" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A3" s="6"/>
+      <c r="B3" s="14" t="s">
+        <v>22</v>
+      </c>
+      <c r="C3" s="15"/>
+      <c r="D3" s="15"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15"/>
+      <c r="G3" s="16"/>
+    </row>
+    <row r="4" spans="1:7" ht="24.95" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A4" s="7"/>
+      <c r="B4" s="14" t="s">
+        <v>23</v>
+      </c>
+      <c r="C4" s="15"/>
+      <c r="D4" s="15"/>
+      <c r="E4" s="15"/>
+      <c r="F4" s="15"/>
+      <c r="G4" s="16"/>
+    </row>
+    <row r="5" spans="1:7" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A5" s="29"/>
+      <c r="B5" s="30"/>
+      <c r="C5" s="30"/>
+      <c r="D5" s="30"/>
+      <c r="E5" s="30"/>
+      <c r="F5" s="30"/>
+      <c r="G5" s="31"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="27" t="s">
+        <v>0</v>
+      </c>
+      <c r="B6" s="20"/>
+      <c r="C6" s="21"/>
+      <c r="D6" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="E6" s="17"/>
-      <c r="F6" s="17"/>
-      <c r="G6" s="18"/>
-    </row>
-    <row r="7" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A7" s="20"/>
-      <c r="B7" s="20"/>
-      <c r="C7" s="21"/>
-      <c r="D7" s="19"/>
-      <c r="E7" s="20"/>
-      <c r="F7" s="20"/>
-      <c r="G7" s="21"/>
-    </row>
-    <row r="8" spans="1:7" x14ac:dyDescent="0.35">
+      <c r="E6" s="20"/>
+      <c r="F6" s="20"/>
+      <c r="G6" s="21"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="23"/>
+      <c r="B7" s="23"/>
+      <c r="C7" s="24"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="23"/>
+      <c r="F7" s="23"/>
+      <c r="G7" s="24"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A8" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="B8" s="10" t="s">
-        <v>23</v>
-      </c>
-      <c r="C8" s="15"/>
-      <c r="D8" s="8" t="s">
+      <c r="B8" s="17" t="s">
+        <v>18</v>
+      </c>
+      <c r="C8" s="18"/>
+      <c r="D8" s="25" t="s">
+        <v>24</v>
+      </c>
+      <c r="E8" s="26"/>
+      <c r="F8" s="17">
+        <v>0</v>
+      </c>
+      <c r="G8" s="28"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B9" s="17" t="s">
+        <v>19</v>
+      </c>
+      <c r="C9" s="18"/>
+      <c r="D9" s="25" t="s">
+        <v>25</v>
+      </c>
+      <c r="E9" s="26"/>
+      <c r="F9" s="17">
+        <v>0</v>
+      </c>
+      <c r="G9" s="28"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="B10" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="C10" s="18"/>
+      <c r="D10" s="25" t="s">
+        <v>16</v>
+      </c>
+      <c r="E10" s="26"/>
+      <c r="F10" s="17">
+        <v>0</v>
+      </c>
+      <c r="G10" s="28"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="B11" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="C11" s="18"/>
+      <c r="D11" s="25" t="s">
+        <v>17</v>
+      </c>
+      <c r="E11" s="26"/>
+      <c r="F11" s="17">
+        <v>0</v>
+      </c>
+      <c r="G11" s="28"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E8" s="9"/>
-      <c r="F8" s="10">
-        <v>0</v>
-      </c>
-      <c r="G8" s="11"/>
-    </row>
-    <row r="9" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A9" s="1" t="s">
+      <c r="B12" s="17">
+        <v>0</v>
+      </c>
+      <c r="C12" s="32"/>
+      <c r="D12" s="25" t="s">
+        <v>26</v>
+      </c>
+      <c r="E12" s="26"/>
+      <c r="F12" s="17">
+        <v>0</v>
+      </c>
+      <c r="G12" s="28"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="B9" s="10" t="s">
-        <v>24</v>
-      </c>
-      <c r="C9" s="15"/>
-      <c r="D9" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="E9" s="9"/>
-      <c r="F9" s="10">
-        <v>0</v>
-      </c>
-      <c r="G9" s="11"/>
-    </row>
-    <row r="10" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A10" s="1" t="s">
+      <c r="B13" s="17">
+        <v>0</v>
+      </c>
+      <c r="C13" s="32"/>
+      <c r="D13" s="33" t="s">
+        <v>15</v>
+      </c>
+      <c r="E13" s="33"/>
+      <c r="F13" s="17">
+        <v>0</v>
+      </c>
+      <c r="G13" s="34"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="2" t="s">
         <v>8</v>
       </c>
-      <c r="B10" s="10" t="s">
-        <v>25</v>
-      </c>
-      <c r="C10" s="15"/>
-      <c r="D10" s="8" t="s">
-        <v>21</v>
-      </c>
-      <c r="E10" s="9"/>
-      <c r="F10" s="10">
-        <v>0</v>
-      </c>
-      <c r="G10" s="11"/>
-    </row>
-    <row r="11" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A11" s="1" t="s">
+      <c r="B14" s="2" t="s">
         <v>9</v>
       </c>
-      <c r="B11" s="10" t="s">
-        <v>26</v>
-      </c>
-      <c r="C11" s="15"/>
-      <c r="D11" s="8" t="s">
-        <v>22</v>
-      </c>
-      <c r="E11" s="9"/>
-      <c r="F11" s="10">
-        <v>0</v>
-      </c>
-      <c r="G11" s="11"/>
-    </row>
-    <row r="12" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A12" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="B12" s="10">
-        <v>0</v>
-      </c>
-      <c r="C12" s="12"/>
-      <c r="D12" s="8" t="s">
-        <v>20</v>
-      </c>
-      <c r="E12" s="9"/>
-      <c r="F12" s="10">
-        <v>0</v>
-      </c>
-      <c r="G12" s="11"/>
-    </row>
-    <row r="13" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A13" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="B13" s="10">
-        <v>0</v>
-      </c>
-      <c r="C13" s="12"/>
-      <c r="D13" s="13" t="s">
-        <v>19</v>
-      </c>
-      <c r="E13" s="13"/>
-      <c r="F13" s="10">
-        <v>0</v>
-      </c>
-      <c r="G13" s="14"/>
-    </row>
-    <row r="14" spans="1:7" x14ac:dyDescent="0.35">
-      <c r="A14" s="2" t="s">
+      <c r="C14" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="D14" s="2" t="s">
         <v>10</v>
       </c>
-      <c r="B14" s="2" t="s">
+      <c r="E14" s="2" t="s">
         <v>11</v>
       </c>
-      <c r="C14" s="2" t="s">
+      <c r="F14" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G14" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="D14" s="2" t="s">
-        <v>13</v>
-      </c>
-      <c r="E14" s="2" t="s">
-        <v>14</v>
-      </c>
-      <c r="F14" s="2" t="s">
-        <v>18</v>
-      </c>
-      <c r="G14" s="2" t="s">
-        <v>15</v>
-      </c>
-    </row>
-    <row r="15" spans="1:7" x14ac:dyDescent="0.35">
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A15" s="4">
         <v>44166</v>
       </c>
       <c r="B15" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C15">
         <v>0</v>
@@ -1077,12 +1077,12 @@
         <v>0</v>
       </c>
     </row>
-    <row r="16" spans="1:7" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
       <c r="A16" s="4">
         <v>44180</v>
       </c>
       <c r="B16" s="3" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="C16">
         <v>0</v>
@@ -1099,6 +1099,18 @@
     </row>
   </sheetData>
   <mergeCells count="25">
+    <mergeCell ref="F10:G10"/>
+    <mergeCell ref="F11:G11"/>
+    <mergeCell ref="B10:C10"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="B11:C11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="F12:G12"/>
+    <mergeCell ref="B12:C12"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="F13:G13"/>
     <mergeCell ref="A1:A4"/>
     <mergeCell ref="B1:G2"/>
     <mergeCell ref="B3:G3"/>
@@ -1112,18 +1124,6 @@
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="F9:G9"/>
     <mergeCell ref="A5:G5"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="F12:G12"/>
-    <mergeCell ref="B12:C12"/>
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="F13:G13"/>
-    <mergeCell ref="F10:G10"/>
-    <mergeCell ref="F11:G11"/>
-    <mergeCell ref="B10:C10"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="B11:C11"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>

</xml_diff>